<commit_message>
them danh sach phan cung
</commit_message>
<xml_diff>
--- a/Checklist_du_an_EMC_ca_nhan.xlsx
+++ b/Checklist_du_an_EMC_ca_nhan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\project\EMC_prj\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{325DC0A8-27E3-413A-A87F-452865823564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A642856-55EC-4565-BAEB-2A3D60444552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1597" uniqueCount="774">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1597" uniqueCount="775">
   <si>
     <t>BẢNG ĐIỀU KHIỂN TIẾN ĐỘ DỰ ÁN EMC - 1 NGƯỜI THỰC HIỆN</t>
   </si>
@@ -2359,6 +2359,9 @@
   </si>
   <si>
     <t xml:space="preserve">Chỉ cấm Modul cắm </t>
+  </si>
+  <si>
+    <t>— Không áp dụng</t>
   </si>
 </sst>
 </file>
@@ -3459,7 +3462,7 @@
       <c r="B13" s="56"/>
       <c r="C13" s="57">
         <f>COUNTIF(Checklist!$G$5:$G$134,"☑ Hoàn thành")</f>
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="D13" s="57"/>
       <c r="E13" s="58">
@@ -3502,7 +3505,7 @@
       </c>
       <c r="C16" s="61">
         <f>IFERROR(SUM(Checklist!$H$5:$H$134)/(COUNTIF(Checklist!$A$5:$A$134,"&lt;&gt;")-COUNTIF(Checklist!$G$5:$G$134,"— Không áp dụng")),0)</f>
-        <v>4.6153846153846156E-2</v>
+        <v>0.16279069767441862</v>
       </c>
       <c r="D16" s="61"/>
       <c r="E16" s="61"/>
@@ -3519,7 +3522,7 @@
       </c>
       <c r="C17" s="54">
         <f>COUNTIF(Checklist!$G$5:$G$134,"— Không áp dụng")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="54"/>
       <c r="E17" s="54"/>
@@ -3599,7 +3602,7 @@
       </c>
       <c r="C21" s="9">
         <f>COUNTIFS(Checklist!$B$5:$B$134,A21,Checklist!$G$5:$G$134,"☑ Hoàn thành")</f>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D21" s="9">
         <f>COUNTIFS(Checklist!$B$5:$B$134,A21,Checklist!$G$5:$G$134,"◐ Đang làm")</f>
@@ -3607,7 +3610,7 @@
       </c>
       <c r="E21" s="10">
         <f>IFERROR(SUMIF(Checklist!$B$5:$B$134,A21,Checklist!$H$5:$H$134)/(COUNTIF(Checklist!$B$5:$B$134,A21)-COUNTIFS(Checklist!$B$5:$B$134,A21,Checklist!$G$5:$G$134,"— Không áp dụng")),0)</f>
-        <v>0.1</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="11" t="s">
@@ -3655,7 +3658,7 @@
       </c>
       <c r="C23" s="9">
         <f>COUNTIFS(Checklist!$B$5:$B$134,A23,Checklist!$G$5:$G$134,"☑ Hoàn thành")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D23" s="9">
         <f>COUNTIFS(Checklist!$B$5:$B$134,A23,Checklist!$G$5:$G$134,"◐ Đang làm")</f>
@@ -3663,7 +3666,7 @@
       </c>
       <c r="E23" s="10">
         <f>IFERROR(SUMIF(Checklist!$B$5:$B$134,A23,Checklist!$H$5:$H$134)/(COUNTIF(Checklist!$B$5:$B$134,A23)-COUNTIFS(Checklist!$B$5:$B$134,A23,Checklist!$G$5:$G$134,"— Không áp dụng")),0)</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="13" t="s">
@@ -4469,11 +4472,11 @@
         <v>58</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H10" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" s="24"/>
       <c r="J10" s="14" t="s">
@@ -4509,11 +4512,11 @@
         <v>58</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H11" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11" s="24"/>
       <c r="J11" s="14" t="s">
@@ -4589,11 +4592,11 @@
         <v>58</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H13" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="24"/>
       <c r="J13" s="14" t="s">
@@ -4629,7 +4632,7 @@
         <v>69</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>59</v>
+        <v>774</v>
       </c>
       <c r="H14" s="17">
         <f t="shared" si="0"/>
@@ -4709,11 +4712,11 @@
         <v>58</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H16" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" s="24"/>
       <c r="J16" s="14" t="s">
@@ -4749,11 +4752,11 @@
         <v>58</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H17" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17" s="24"/>
       <c r="J17" s="14" t="s">
@@ -4789,11 +4792,11 @@
         <v>58</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H18" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18" s="24"/>
       <c r="J18" s="14" t="s">
@@ -4829,11 +4832,11 @@
         <v>58</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H19" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" s="24"/>
       <c r="J19" s="14" t="s">
@@ -5189,11 +5192,11 @@
         <v>58</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H28" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" s="24"/>
       <c r="J28" s="14" t="s">
@@ -5229,11 +5232,11 @@
         <v>58</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H29" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" s="24"/>
       <c r="J29" s="14" t="s">
@@ -5269,11 +5272,11 @@
         <v>58</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H30" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" s="24"/>
       <c r="J30" s="14" t="s">
@@ -5309,11 +5312,11 @@
         <v>58</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H31" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31" s="24"/>
       <c r="J31" s="14" t="s">
@@ -5349,11 +5352,11 @@
         <v>58</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H32" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" s="24"/>
       <c r="J32" s="14" t="s">
@@ -5389,11 +5392,11 @@
         <v>58</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H33" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I33" s="24"/>
       <c r="J33" s="14" t="s">
@@ -5429,11 +5432,11 @@
         <v>69</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H34" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I34" s="24"/>
       <c r="J34" s="14" t="s">
@@ -5549,11 +5552,11 @@
         <v>58</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>59</v>
+        <v>772</v>
       </c>
       <c r="H37" s="17">
         <f t="shared" ref="H37:H68" si="2">IF(G37="☑ Hoàn thành",1,IF(G37="◐ Đang làm",0.5,IF(G37="⚠ Bị chặn",0.25,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" s="24"/>
       <c r="J37" s="14" t="s">

</xml_diff>